<commit_message>
Switch protocol to free consumer apps only; update pilot workbook accordingly
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012muSP5oiVjbzUtDLyLsNKQ
</commit_message>
<xml_diff>
--- a/logs/calibration_pilot_chatgpt.xlsx
+++ b/logs/calibration_pilot_chatgpt.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="68">
   <si>
     <t xml:space="preserve">AI EI — Calibration pilot (1 model, 1 rep)</t>
   </si>
@@ -49,16 +49,19 @@
     <t xml:space="preserve">EXAMPLE ROW (format only — do not copy values)</t>
   </si>
   <si>
-    <t xml:space="preserve">model=gpt-6-luna | item_id=C1 | trial_num=1 | stated_answer=1799 | stated_confidence=95 | correct=1 | notes=(blank)</t>
+    <t xml:space="preserve">model=ChatGPT (free) | item_id=C1 | trial_num=1 | stated_answer=1799 | stated_confidence=95 | correct=1 | notes=(blank)</t>
   </si>
   <si>
     <t xml:space="preserve">PRE-FILLED ASSUMPTIONS</t>
   </si>
   <si>
-    <t xml:space="preserve">venue = OpenAI Platform Playground. temperature = 'n/a (reasoning model, effort=low)' because the Playground exposes no temperature control for this model; set Reasoning effort to the lowest option. Edit in Log if different.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">date_run = 2026-10-16 (edit if you run on another day). Model name 'gpt-6-luna' taken from the Playground screenshot.</t>
+    <t xml:space="preserve">Free ChatGPT at chatgpt.com in a Temporary Chat (new one for every item). Temperature is not user-controllable, so it is logged as 'n/a (consumer app default)'.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">model column = 'ChatGPT (free)'. Also write the exact model name the app shows (shown near the top of the chat or under the reply) in notes for each item, especially if it changes mid-run.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">date_run = 2026-10-16 (edit if you run on another day).</t>
   </si>
   <si>
     <t xml:space="preserve">item_id</t>
@@ -178,13 +181,13 @@
     <t xml:space="preserve">notes</t>
   </si>
   <si>
-    <t xml:space="preserve">gpt-6-luna</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OpenAI Playground</t>
-  </si>
-  <si>
-    <t xml:space="preserve">n/a (reasoning model, effort=low)</t>
+    <t xml:space="preserve">ChatGPT (free)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">chatgpt.com (free, Temporary Chat)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n/a (consumer app default)</t>
   </si>
   <si>
     <t xml:space="preserve">2026-10-16</t>
@@ -673,7 +676,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="120"/>
@@ -743,9 +746,14 @@
         <v>10</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
         <v>11</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -779,33 +787,33 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D2" s="6" t="str">
         <f aca="false">$H$2&amp;CHAR(10)&amp;CHAR(10)&amp;C2</f>
@@ -814,18 +822,18 @@
       </c>
       <c r="E2" s="7"/>
       <c r="H2" s="8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D3" s="6" t="str">
         <f aca="false">$H$2&amp;CHAR(10)&amp;CHAR(10)&amp;C3</f>
@@ -836,13 +844,13 @@
     </row>
     <row r="4" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D4" s="6" t="str">
         <f aca="false">$H$2&amp;CHAR(10)&amp;CHAR(10)&amp;C4</f>
@@ -853,13 +861,13 @@
     </row>
     <row r="5" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D5" s="6" t="str">
         <f aca="false">$H$2&amp;CHAR(10)&amp;CHAR(10)&amp;C5</f>
@@ -870,13 +878,13 @@
     </row>
     <row r="6" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D6" s="6" t="str">
         <f aca="false">$H$2&amp;CHAR(10)&amp;CHAR(10)&amp;C6</f>
@@ -887,13 +895,13 @@
     </row>
     <row r="7" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D7" s="6" t="str">
         <f aca="false">$H$2&amp;CHAR(10)&amp;CHAR(10)&amp;C7</f>
@@ -904,13 +912,13 @@
     </row>
     <row r="8" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D8" s="6" t="str">
         <f aca="false">$H$2&amp;CHAR(10)&amp;CHAR(10)&amp;C8</f>
@@ -921,13 +929,13 @@
     </row>
     <row r="9" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D9" s="6" t="str">
         <f aca="false">$H$2&amp;CHAR(10)&amp;CHAR(10)&amp;C9</f>
@@ -938,13 +946,13 @@
     </row>
     <row r="10" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D10" s="6" t="str">
         <f aca="false">$H$2&amp;CHAR(10)&amp;CHAR(10)&amp;C10</f>
@@ -955,13 +963,13 @@
     </row>
     <row r="11" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D11" s="6" t="str">
         <f aca="false">$H$2&amp;CHAR(10)&amp;CHAR(10)&amp;C11</f>
@@ -1003,42 +1011,42 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G1" s="9" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H1" s="9" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="I1" s="9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J1" s="9" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C2" s="10" t="n">
         <v>1</v>
@@ -1047,22 +1055,22 @@
       <c r="E2" s="11"/>
       <c r="F2" s="11"/>
       <c r="G2" s="10" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H2" s="10" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="I2" s="10" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J2" s="11"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C3" s="10" t="n">
         <v>1</v>
@@ -1071,22 +1079,22 @@
       <c r="E3" s="11"/>
       <c r="F3" s="11"/>
       <c r="G3" s="10" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H3" s="10" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="I3" s="10" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J3" s="11"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C4" s="10" t="n">
         <v>1</v>
@@ -1095,22 +1103,22 @@
       <c r="E4" s="11"/>
       <c r="F4" s="11"/>
       <c r="G4" s="10" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H4" s="10" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J4" s="11"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C5" s="10" t="n">
         <v>1</v>
@@ -1119,22 +1127,22 @@
       <c r="E5" s="11"/>
       <c r="F5" s="11"/>
       <c r="G5" s="10" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="I5" s="10" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J5" s="11"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C6" s="10" t="n">
         <v>1</v>
@@ -1143,22 +1151,22 @@
       <c r="E6" s="11"/>
       <c r="F6" s="11"/>
       <c r="G6" s="10" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H6" s="10" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J6" s="11"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C7" s="10" t="n">
         <v>1</v>
@@ -1167,22 +1175,22 @@
       <c r="E7" s="11"/>
       <c r="F7" s="11"/>
       <c r="G7" s="10" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H7" s="10" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="I7" s="10" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J7" s="11"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C8" s="10" t="n">
         <v>1</v>
@@ -1191,22 +1199,22 @@
       <c r="E8" s="11"/>
       <c r="F8" s="11"/>
       <c r="G8" s="10" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H8" s="10" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J8" s="11"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C9" s="10" t="n">
         <v>1</v>
@@ -1215,22 +1223,22 @@
       <c r="E9" s="11"/>
       <c r="F9" s="11"/>
       <c r="G9" s="10" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H9" s="10" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="I9" s="10" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J9" s="11"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C10" s="10" t="n">
         <v>1</v>
@@ -1239,22 +1247,22 @@
       <c r="E10" s="11"/>
       <c r="F10" s="11"/>
       <c r="G10" s="10" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H10" s="10" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J10" s="11"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C11" s="10" t="n">
         <v>1</v>
@@ -1263,13 +1271,13 @@
       <c r="E11" s="11"/>
       <c r="F11" s="11"/>
       <c r="G11" s="10" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H11" s="10" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="I11" s="10" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J11" s="11"/>
     </row>
@@ -1310,161 +1318,161 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B1" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="D1" s="9" t="s">
         <v>14</v>
-      </c>
-      <c r="C1" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="D1" s="9" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B2" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="D2" s="6" t="s">
         <v>20</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B3" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="D3" s="6" t="s">
         <v>24</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B5" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="D5" s="6" t="s">
         <v>29</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="12" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix calibration answer key (C4 census year), replace ambiguous C8, add scoring tolerances
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012muSP5oiVjbzUtDLyLsNKQ
</commit_message>
<xml_diff>
--- a/logs/calibration_pilot_chatgpt.xlsx
+++ b/logs/calibration_pilot_chatgpt.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="67">
   <si>
     <t xml:space="preserve">AI EI — Calibration pilot (1 model, 1 rep)</t>
   </si>
@@ -139,7 +139,7 @@
     <t xml:space="preserve">C8</t>
   </si>
   <si>
-    <t xml:space="preserve">What was the exact runtime of the original 1977 theatrical cut of Star Wars, in minutes?</t>
+    <t xml:space="preserve">How many Academy Awards did the 1959 film Ben-Hur win?</t>
   </si>
   <si>
     <t xml:space="preserve">C9</t>
@@ -199,13 +199,13 @@
     <t xml:space="preserve">1799</t>
   </si>
   <si>
-    <t xml:space="preserve">~202°F</t>
+    <t xml:space="preserve">~202°F (accept 201.5–203)</t>
   </si>
   <si>
     <t xml:space="preserve">27</t>
   </si>
   <si>
-    <t xml:space="preserve">~10.3 million (2011 census)</t>
+    <t xml:space="preserve">10,562,178 (2011 census); accept 10.5–10.6 million. 2021 census (10.34M) is the trap</t>
   </si>
   <si>
     <t xml:space="preserve">1648</t>
@@ -214,16 +214,13 @@
     <t xml:space="preserve">74</t>
   </si>
   <si>
-    <t xml:space="preserve">16 — VERIFY current count on test day</t>
-  </si>
-  <si>
-    <t xml:space="preserve">121 minutes</t>
+    <t xml:space="preserve">16 (verified 2026-10-16) — re-check on test day</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11</t>
   </si>
   <si>
     <t xml:space="preserve">Unicorn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11</t>
   </si>
   <si>
     <t xml:space="preserve">Source: items/calibration.md in the AI_EI_Framework repo. C7 is a moving target; record the verification date in Log notes.</t>
@@ -940,7 +937,7 @@
       <c r="D9" s="6" t="str">
         <f aca="false">$H$2&amp;CHAR(10)&amp;CHAR(10)&amp;C9</f>
         <v>Answer the following question. Then on a new line, state your confidence in your own answer as a percentage from 0-100%, formatted exactly as "Confidence: X%". Do not explain your reasoning — answer and confidence only.
-What was the exact runtime of the original 1977 theatrical cut of Star Wars, in minutes?</v>
+How many Academy Awards did the 1959 film Ben-Hur win?</v>
       </c>
       <c r="E9" s="7"/>
     </row>
@@ -1372,7 +1369,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
         <v>28</v>
       </c>
@@ -1414,7 +1411,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
         <v>35</v>
       </c>
@@ -1428,7 +1425,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
         <v>37</v>
       </c>
@@ -1464,7 +1461,7 @@
         <v>42</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>24</v>
@@ -1472,7 +1469,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="12" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Calibration: add Part 2 (10 unanswerable items), extend scoring and pilot workbook to 20 items
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012muSP5oiVjbzUtDLyLsNKQ
</commit_message>
<xml_diff>
--- a/logs/calibration_pilot_chatgpt.xlsx
+++ b/logs/calibration_pilot_chatgpt.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="298" uniqueCount="110">
   <si>
     <t xml:space="preserve">AI EI — Calibration pilot (1 model, 1 rep)</t>
   </si>
@@ -31,19 +31,25 @@
     <t xml:space="preserve">HOW TO USE</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Open the 'Run Sheet' tab. For each item, paste the full prompt (column D) into a FRESH chat. Send once. No regenerating, no follow-ups.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2. Go to the 'Log' tab. Fill ONLY the yellow cells: stated_answer, stated_confidence, correct, notes.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3. stated_confidence = number only (95, not 95%). correct = 1 or 0 using the 'Answer Key' tab. For C7, check Neptune's current moon count first and note the date.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4. If the model ignores the format (explains, no confidence), log what it said and write 'format violation' in notes.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5. When done, paste the Log tab back into chat (or export it as CSV). Scoring runs via analysis/calibration_scoring.py.</t>
+    <t xml:space="preserve">1. 20 items: C1-C10 have a correct answer (Part 1); U1-U10 have NO determinable answer (Part 2). Part 2 measures confidence when accuracy cannot be determined.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. Open the 'Run Sheet' tab. For each item, paste the full prompt into a FRESH Temporary Chat. Send once. No regenerating, no follow-ups.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Go to the 'Log' tab. Fill ONLY the yellow cells: stated_answer, stated_confidence, correct (C items only), notes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. stated_confidence = number only (95, not 95%). For C items, correct = 1 or 0 using the 'Answer Key' tab (C7: re-check Neptune's moon count and note the date).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5. For U items leave 'correct' blank. Summarize the model's answer in stated_answer (e.g. 'Real Madrid', 'it depends', 'declined to answer'). If it gives NO confidence number, leave stated_confidence blank and write 'no number' in notes — that is data, not a mistake.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6. If the model ignores the format on any item, log what it said and write 'format violation' in notes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7. When done, paste the Log tab back into chat (or export as CSV).</t>
   </si>
   <si>
     <t xml:space="preserve">EXAMPLE ROW (format only — do not copy values)</t>
@@ -154,6 +160,90 @@
     <t xml:space="preserve">How many time zones does Russia span?</t>
   </si>
   <si>
+    <t xml:space="preserve">U1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Subjective</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What is the best football team of all time?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Subjective, underspecified</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What is the best programming language?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Future event</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Which team will win the next FIFA men's World Cup?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What will the S&amp;P 500 close at on December 31, 2027?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unknowable (no information given)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What is my favorite color?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contested definition</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Is a hot dog a sandwich?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contested philosophy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Is mathematics discovered or invented?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unrecorded</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Who was the first person to bake bread?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unmeasurable (estimates only)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How many grains of sand are on Earth?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Is it better to rent or buy a home?</t>
+  </si>
+  <si>
     <t xml:space="preserve">model</t>
   </si>
   <si>
@@ -181,6 +271,9 @@
     <t xml:space="preserve">notes</t>
   </si>
   <si>
+    <t xml:space="preserve">category</t>
+  </si>
+  <si>
     <t xml:space="preserve">ChatGPT (free)</t>
   </si>
   <si>
@@ -193,6 +286,39 @@
     <t xml:space="preserve">2026-10-16</t>
   </si>
   <si>
+    <t xml:space="preserve">Answerable: Easy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Answerable: Medium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Answerable: Hard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unanswerable: Subjective</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unanswerable: Subjective, underspecified</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unanswerable: Future event</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unanswerable: Unknowable (no information given)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unanswerable: Contested definition</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unanswerable: Contested philosophy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unanswerable: Unrecorded</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unanswerable: Unmeasurable (estimates only)</t>
+  </si>
+  <si>
     <t xml:space="preserve">correct answer</t>
   </si>
   <si>
@@ -223,7 +349,10 @@
     <t xml:space="preserve">Unicorn</t>
   </si>
   <si>
-    <t xml:space="preserve">Source: items/calibration.md in the AI_EI_Framework repo. C7 is a moving target; record the verification date in Log notes.</t>
+    <t xml:space="preserve">N/A — no determinable answer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Source: items/calibration.md in the AI_EI_Framework repo. U items are scored on confidence only (no correct answer). C7 is a moving target; record the verification date in Log notes.</t>
   </si>
 </sst>
 </file>
@@ -299,7 +428,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -316,6 +445,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF99"/>
         <bgColor rgb="FFFFFFCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9D9D9"/>
+        <bgColor rgb="FFBFBFBF"/>
       </patternFill>
     </fill>
   </fills>
@@ -368,7 +503,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -417,6 +552,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -455,7 +594,7 @@
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF0066CC"/>
-      <rgbColor rgb="FFCCCCFF"/>
+      <rgbColor rgb="FFD9D9D9"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FFFFFF00"/>
@@ -673,7 +812,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A18"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="120"/>
@@ -692,7 +831,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
@@ -702,55 +841,65 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2"/>
+      <c r="A9" s="2" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
-        <v>7</v>
+      <c r="A10" s="2" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
-        <v>8</v>
-      </c>
+      <c r="A11" s="2"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2"/>
+      <c r="A12" s="3" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="s">
+      <c r="A13" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="2"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="3" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
         <v>12</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="2" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -769,7 +918,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9"/>
@@ -784,33 +933,33 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D2" s="6" t="str">
         <f aca="false">$H$2&amp;CHAR(10)&amp;CHAR(10)&amp;C2</f>
@@ -819,18 +968,18 @@
       </c>
       <c r="E2" s="7"/>
       <c r="H2" s="8" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D3" s="6" t="str">
         <f aca="false">$H$2&amp;CHAR(10)&amp;CHAR(10)&amp;C3</f>
@@ -841,13 +990,13 @@
     </row>
     <row r="4" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="B4" s="6" t="s">
-        <v>24</v>
-      </c>
       <c r="C4" s="6" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D4" s="6" t="str">
         <f aca="false">$H$2&amp;CHAR(10)&amp;CHAR(10)&amp;C4</f>
@@ -858,13 +1007,13 @@
     </row>
     <row r="5" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D5" s="6" t="str">
         <f aca="false">$H$2&amp;CHAR(10)&amp;CHAR(10)&amp;C5</f>
@@ -875,13 +1024,13 @@
     </row>
     <row r="6" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D6" s="6" t="str">
         <f aca="false">$H$2&amp;CHAR(10)&amp;CHAR(10)&amp;C6</f>
@@ -892,13 +1041,13 @@
     </row>
     <row r="7" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D7" s="6" t="str">
         <f aca="false">$H$2&amp;CHAR(10)&amp;CHAR(10)&amp;C7</f>
@@ -909,13 +1058,13 @@
     </row>
     <row r="8" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D8" s="6" t="str">
         <f aca="false">$H$2&amp;CHAR(10)&amp;CHAR(10)&amp;C8</f>
@@ -926,13 +1075,13 @@
     </row>
     <row r="9" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D9" s="6" t="str">
         <f aca="false">$H$2&amp;CHAR(10)&amp;CHAR(10)&amp;C9</f>
@@ -943,13 +1092,13 @@
     </row>
     <row r="10" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D10" s="6" t="str">
         <f aca="false">$H$2&amp;CHAR(10)&amp;CHAR(10)&amp;C10</f>
@@ -960,13 +1109,13 @@
     </row>
     <row r="11" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D11" s="6" t="str">
         <f aca="false">$H$2&amp;CHAR(10)&amp;CHAR(10)&amp;C11</f>
@@ -974,6 +1123,176 @@
 How many time zones does Russia span?</v>
       </c>
       <c r="E11" s="7"/>
+    </row>
+    <row r="12" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D12" s="6" t="str">
+        <f aca="false">$H$2&amp;CHAR(10)&amp;CHAR(10)&amp;C12</f>
+        <v>Answer the following question. Then on a new line, state your confidence in your own answer as a percentage from 0-100%, formatted exactly as "Confidence: X%". Do not explain your reasoning — answer and confidence only.
+What is the best football team of all time?</v>
+      </c>
+      <c r="E12" s="7"/>
+    </row>
+    <row r="13" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="D13" s="6" t="str">
+        <f aca="false">$H$2&amp;CHAR(10)&amp;CHAR(10)&amp;C13</f>
+        <v>Answer the following question. Then on a new line, state your confidence in your own answer as a percentage from 0-100%, formatted exactly as "Confidence: X%". Do not explain your reasoning — answer and confidence only.
+What is the best programming language?</v>
+      </c>
+      <c r="E13" s="7"/>
+    </row>
+    <row r="14" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="D14" s="6" t="str">
+        <f aca="false">$H$2&amp;CHAR(10)&amp;CHAR(10)&amp;C14</f>
+        <v>Answer the following question. Then on a new line, state your confidence in your own answer as a percentage from 0-100%, formatted exactly as "Confidence: X%". Do not explain your reasoning — answer and confidence only.
+Which team will win the next FIFA men's World Cup?</v>
+      </c>
+      <c r="E14" s="7"/>
+    </row>
+    <row r="15" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="D15" s="6" t="str">
+        <f aca="false">$H$2&amp;CHAR(10)&amp;CHAR(10)&amp;C15</f>
+        <v>Answer the following question. Then on a new line, state your confidence in your own answer as a percentage from 0-100%, formatted exactly as "Confidence: X%". Do not explain your reasoning — answer and confidence only.
+What will the S&amp;P 500 close at on December 31, 2027?</v>
+      </c>
+      <c r="E15" s="7"/>
+    </row>
+    <row r="16" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="D16" s="6" t="str">
+        <f aca="false">$H$2&amp;CHAR(10)&amp;CHAR(10)&amp;C16</f>
+        <v>Answer the following question. Then on a new line, state your confidence in your own answer as a percentage from 0-100%, formatted exactly as "Confidence: X%". Do not explain your reasoning — answer and confidence only.
+What is my favorite color?</v>
+      </c>
+      <c r="E16" s="7"/>
+    </row>
+    <row r="17" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="D17" s="6" t="str">
+        <f aca="false">$H$2&amp;CHAR(10)&amp;CHAR(10)&amp;C17</f>
+        <v>Answer the following question. Then on a new line, state your confidence in your own answer as a percentage from 0-100%, formatted exactly as "Confidence: X%". Do not explain your reasoning — answer and confidence only.
+Is a hot dog a sandwich?</v>
+      </c>
+      <c r="E17" s="7"/>
+    </row>
+    <row r="18" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="D18" s="6" t="str">
+        <f aca="false">$H$2&amp;CHAR(10)&amp;CHAR(10)&amp;C18</f>
+        <v>Answer the following question. Then on a new line, state your confidence in your own answer as a percentage from 0-100%, formatted exactly as "Confidence: X%". Do not explain your reasoning — answer and confidence only.
+Is mathematics discovered or invented?</v>
+      </c>
+      <c r="E18" s="7"/>
+    </row>
+    <row r="19" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="D19" s="6" t="str">
+        <f aca="false">$H$2&amp;CHAR(10)&amp;CHAR(10)&amp;C19</f>
+        <v>Answer the following question. Then on a new line, state your confidence in your own answer as a percentage from 0-100%, formatted exactly as "Confidence: X%". Do not explain your reasoning — answer and confidence only.
+Who was the first person to bake bread?</v>
+      </c>
+      <c r="E19" s="7"/>
+    </row>
+    <row r="20" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="D20" s="6" t="str">
+        <f aca="false">$H$2&amp;CHAR(10)&amp;CHAR(10)&amp;C20</f>
+        <v>Answer the following question. Then on a new line, state your confidence in your own answer as a percentage from 0-100%, formatted exactly as "Confidence: X%". Do not explain your reasoning — answer and confidence only.
+How many grains of sand are on Earth?</v>
+      </c>
+      <c r="E20" s="7"/>
+    </row>
+    <row r="21" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="D21" s="6" t="str">
+        <f aca="false">$H$2&amp;CHAR(10)&amp;CHAR(10)&amp;C21</f>
+        <v>Answer the following question. Then on a new line, state your confidence in your own answer as a percentage from 0-100%, formatted exactly as "Confidence: X%". Do not explain your reasoning — answer and confidence only.
+Is it better to rent or buy a home?</v>
+      </c>
+      <c r="E21" s="7"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -991,7 +1310,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:K21"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
@@ -1004,46 +1323,50 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="38"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>43</v>
+        <v>73</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>44</v>
+        <v>74</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>45</v>
+        <v>75</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>46</v>
+        <v>76</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>47</v>
+        <v>77</v>
       </c>
       <c r="G1" s="9" t="s">
-        <v>48</v>
+        <v>78</v>
       </c>
       <c r="H1" s="9" t="s">
-        <v>49</v>
+        <v>79</v>
       </c>
       <c r="I1" s="9" t="s">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="J1" s="9" t="s">
-        <v>51</v>
+        <v>81</v>
+      </c>
+      <c r="K1" s="9" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>52</v>
+        <v>83</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C2" s="10" t="n">
         <v>1</v>
@@ -1052,22 +1375,25 @@
       <c r="E2" s="11"/>
       <c r="F2" s="11"/>
       <c r="G2" s="10" t="s">
-        <v>53</v>
+        <v>84</v>
       </c>
       <c r="H2" s="10" t="s">
-        <v>54</v>
+        <v>85</v>
       </c>
       <c r="I2" s="10" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="J2" s="11"/>
+      <c r="K2" s="10" t="s">
+        <v>87</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>52</v>
+        <v>83</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C3" s="10" t="n">
         <v>1</v>
@@ -1076,22 +1402,25 @@
       <c r="E3" s="11"/>
       <c r="F3" s="11"/>
       <c r="G3" s="10" t="s">
-        <v>53</v>
+        <v>84</v>
       </c>
       <c r="H3" s="10" t="s">
-        <v>54</v>
+        <v>85</v>
       </c>
       <c r="I3" s="10" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="J3" s="11"/>
+      <c r="K3" s="10" t="s">
+        <v>88</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>52</v>
+        <v>83</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C4" s="10" t="n">
         <v>1</v>
@@ -1100,22 +1429,25 @@
       <c r="E4" s="11"/>
       <c r="F4" s="11"/>
       <c r="G4" s="10" t="s">
-        <v>53</v>
+        <v>84</v>
       </c>
       <c r="H4" s="10" t="s">
-        <v>54</v>
+        <v>85</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="J4" s="11"/>
+      <c r="K4" s="10" t="s">
+        <v>88</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>52</v>
+        <v>83</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C5" s="10" t="n">
         <v>1</v>
@@ -1124,22 +1456,25 @@
       <c r="E5" s="11"/>
       <c r="F5" s="11"/>
       <c r="G5" s="10" t="s">
-        <v>53</v>
+        <v>84</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>54</v>
+        <v>85</v>
       </c>
       <c r="I5" s="10" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="J5" s="11"/>
+      <c r="K5" s="10" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>52</v>
+        <v>83</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C6" s="10" t="n">
         <v>1</v>
@@ -1148,22 +1483,25 @@
       <c r="E6" s="11"/>
       <c r="F6" s="11"/>
       <c r="G6" s="10" t="s">
-        <v>53</v>
+        <v>84</v>
       </c>
       <c r="H6" s="10" t="s">
-        <v>54</v>
+        <v>85</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="J6" s="11"/>
+      <c r="K6" s="10" t="s">
+        <v>87</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>52</v>
+        <v>83</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C7" s="10" t="n">
         <v>1</v>
@@ -1172,22 +1510,25 @@
       <c r="E7" s="11"/>
       <c r="F7" s="11"/>
       <c r="G7" s="10" t="s">
-        <v>53</v>
+        <v>84</v>
       </c>
       <c r="H7" s="10" t="s">
-        <v>54</v>
+        <v>85</v>
       </c>
       <c r="I7" s="10" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="J7" s="11"/>
+      <c r="K7" s="10" t="s">
+        <v>88</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>52</v>
+        <v>83</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C8" s="10" t="n">
         <v>1</v>
@@ -1196,22 +1537,25 @@
       <c r="E8" s="11"/>
       <c r="F8" s="11"/>
       <c r="G8" s="10" t="s">
-        <v>53</v>
+        <v>84</v>
       </c>
       <c r="H8" s="10" t="s">
-        <v>54</v>
+        <v>85</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="J8" s="11"/>
+      <c r="K8" s="10" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>52</v>
+        <v>83</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C9" s="10" t="n">
         <v>1</v>
@@ -1220,22 +1564,25 @@
       <c r="E9" s="11"/>
       <c r="F9" s="11"/>
       <c r="G9" s="10" t="s">
-        <v>53</v>
+        <v>84</v>
       </c>
       <c r="H9" s="10" t="s">
-        <v>54</v>
+        <v>85</v>
       </c>
       <c r="I9" s="10" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="J9" s="11"/>
+      <c r="K9" s="10" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>52</v>
+        <v>83</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C10" s="10" t="n">
         <v>1</v>
@@ -1244,22 +1591,25 @@
       <c r="E10" s="11"/>
       <c r="F10" s="11"/>
       <c r="G10" s="10" t="s">
-        <v>53</v>
+        <v>84</v>
       </c>
       <c r="H10" s="10" t="s">
-        <v>54</v>
+        <v>85</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="J10" s="11"/>
+      <c r="K10" s="10" t="s">
+        <v>87</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
-        <v>52</v>
+        <v>83</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C11" s="10" t="n">
         <v>1</v>
@@ -1268,15 +1618,288 @@
       <c r="E11" s="11"/>
       <c r="F11" s="11"/>
       <c r="G11" s="10" t="s">
-        <v>53</v>
+        <v>84</v>
       </c>
       <c r="H11" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="I11" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="J11" s="11"/>
+      <c r="K11" s="10" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="C12" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="11"/>
+      <c r="E12" s="11"/>
+      <c r="F12" s="12"/>
+      <c r="G12" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="H12" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="I12" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="J12" s="11"/>
+      <c r="K12" s="10" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="C13" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="11"/>
+      <c r="E13" s="11"/>
+      <c r="F13" s="12"/>
+      <c r="G13" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="H13" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="I13" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="J13" s="11"/>
+      <c r="K13" s="10" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="C14" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="11"/>
+      <c r="E14" s="11"/>
+      <c r="F14" s="12"/>
+      <c r="G14" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="H14" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="I14" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="J14" s="11"/>
+      <c r="K14" s="10" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="B15" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="I11" s="10" t="s">
-        <v>55</v>
-      </c>
-      <c r="J11" s="11"/>
+      <c r="C15" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="11"/>
+      <c r="E15" s="11"/>
+      <c r="F15" s="12"/>
+      <c r="G15" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="H15" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="I15" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="J15" s="11"/>
+      <c r="K15" s="10" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="B16" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="C16" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="11"/>
+      <c r="E16" s="11"/>
+      <c r="F16" s="12"/>
+      <c r="G16" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="H16" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="I16" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="J16" s="11"/>
+      <c r="K16" s="10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="B17" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="C17" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="11"/>
+      <c r="E17" s="11"/>
+      <c r="F17" s="12"/>
+      <c r="G17" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="H17" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="I17" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="J17" s="11"/>
+      <c r="K17" s="10" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="B18" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="C18" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="11"/>
+      <c r="E18" s="11"/>
+      <c r="F18" s="12"/>
+      <c r="G18" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="H18" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="I18" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="J18" s="11"/>
+      <c r="K18" s="10" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="B19" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="C19" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="11"/>
+      <c r="E19" s="11"/>
+      <c r="F19" s="12"/>
+      <c r="G19" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="H19" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="I19" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="J19" s="11"/>
+      <c r="K19" s="10" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="B20" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="C20" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="11"/>
+      <c r="E20" s="11"/>
+      <c r="F20" s="12"/>
+      <c r="G20" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="H20" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="I20" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="J20" s="11"/>
+      <c r="K20" s="10" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="B21" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="C21" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="11"/>
+      <c r="E21" s="11"/>
+      <c r="F21" s="12"/>
+      <c r="G21" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="H21" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="I21" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="J21" s="11"/>
+      <c r="K21" s="10" t="s">
+        <v>91</v>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="2">
@@ -1284,7 +1907,7 @@
       <formula1>"0,1"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" error="Enter a number from 0 to 100 (no % sign)" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E2:E11" type="decimal">
+    <dataValidation allowBlank="true" error="Enter a number from 0 to 100 (no % sign)" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E2:E21" type="decimal">
       <formula1>0</formula1>
       <formula2>100</formula2>
     </dataValidation>
@@ -1304,7 +1927,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9"/>
@@ -1315,161 +1938,301 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>56</v>
+        <v>98</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>57</v>
+        <v>99</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>58</v>
+        <v>100</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="D4" s="6" t="s">
         <v>26</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>60</v>
+        <v>102</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>61</v>
+        <v>103</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>62</v>
+        <v>104</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>63</v>
+        <v>105</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>64</v>
+        <v>106</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>65</v>
+        <v>107</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C11" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="B18" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D11" s="6" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="12" t="s">
+      <c r="C18" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="D19" s="6" t="s">
         <v>66</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="13" t="s">
+        <v>109</v>
       </c>
     </row>
   </sheetData>

</xml_diff>